<commit_message>
v0.6 - Add command line month filtering
</commit_message>
<xml_diff>
--- a/data/input/january.xlsx
+++ b/data/input/january.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/64bab628b403b612/Belgeler/GitHub/ExcelReporter/data/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="73" documentId="11_F25DC773A252ABDACC1048EAB19C73525BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8BEE5059-9E8F-4F9A-B690-324564155858}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="11_F25DC773A252ABDACC1048EAB19C73525BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB755834-1251-4191-BE3B-70A7C6990753}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>